<commit_message>
add country based fee table
</commit_message>
<xml_diff>
--- a/public/course-import-template.xlsx
+++ b/public/course-import-template.xlsx
@@ -397,14 +397,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:AF2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="18.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="18.83203125" customWidth="1"/>
+    <col min="24" max="24" width="18.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
+    <col min="26" max="26" width="18.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="18.83203125" customWidth="1"/>
+    <col min="29" max="29" width="18.83203125" customWidth="1"/>
+    <col min="30" max="30" width="18.83203125" customWidth="1"/>
+    <col min="31" max="31" width="18.83203125" customWidth="1"/>
+    <col min="32" max="32" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Course Name</v>
       </c>
       <c r="B1" t="str">
-        <v>Mentor Name</v>
+        <v>Mentor</v>
       </c>
       <c r="C1" t="str">
         <v>Description</v>
@@ -413,205 +447,191 @@
         <v>Service Type</v>
       </c>
       <c r="E1" t="str">
+        <v>Level</v>
+      </c>
+      <c r="F1" t="str">
         <v>Start Date</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>End Date</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Duration</v>
       </c>
-      <c r="H1" t="str">
-        <v>Fee</v>
-      </c>
       <c r="I1" t="str">
-        <v>Discount</v>
+        <v>Language</v>
       </c>
       <c r="J1" t="str">
-        <v>Final Price</v>
+        <v>Start Time</v>
       </c>
       <c r="K1" t="str">
-        <v>Level</v>
+        <v>End Time</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Batch Type</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Course Type</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Fee (USA)</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Discount (USA)</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Price (USA)</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Fee (Canadian)</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Discount (Canadian)</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Price (Canadian)</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Fee (Europe)</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Discount (Europe)</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Price (Europe)</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Fee (India)</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Discount (India)</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Price (India)</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Fee (Australia)</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Discount (Australia)</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Price (Australia)</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Fee (Singapore)</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Discount (Singapore)</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Price (Singapore)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Gen AI course</v>
+        <v>Advanced Python</v>
       </c>
       <c r="B2" t="str">
-        <v>Harish Singh</v>
+        <v>John Doe</v>
       </c>
       <c r="C2" t="str">
-        <v>Intro to Gen AI with tools</v>
+        <v>Comprehensive Python course covering advanced topics.</v>
       </c>
       <c r="D2" t="str">
-        <v>Generative AI</v>
+        <v>Agile</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-02-25</v>
+        <v>Advanced</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-02-28</v>
-      </c>
-      <c r="G2">
-        <v>5</v>
+        <v>2026-03-01</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-03-30</v>
       </c>
       <c r="H2">
-        <v>18990</v>
-      </c>
-      <c r="I2">
-        <v>18</v>
-      </c>
-      <c r="J2">
-        <v>15571.8</v>
+        <v>30</v>
+      </c>
+      <c r="I2" t="str">
+        <v>English</v>
+      </c>
+      <c r="J2" t="str">
+        <v>10:00</v>
       </c>
       <c r="K2" t="str">
-        <v>Intermediate</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Agile Fundamentals</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Jane Smith</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Agile basics and scrum</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Agile</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-03-05</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-03-20</v>
-      </c>
-      <c r="G3">
-        <v>20</v>
-      </c>
-      <c r="H3">
-        <v>8990</v>
-      </c>
-      <c r="I3">
+        <v>12:00</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Weekdays</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Online</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2">
+        <v>500</v>
+      </c>
+      <c r="P2">
         <v>10</v>
       </c>
-      <c r="J3">
-        <v>8091</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Beginner</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>SAFe Practitioner</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Ravi Kumar</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Scaled Agile framework</v>
-      </c>
-      <c r="D4" t="str">
-        <v>SAFe</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2026-04-01</v>
-      </c>
-      <c r="F4" t="str">
-        <v>2026-04-10</v>
-      </c>
-      <c r="G4">
-        <v>30</v>
-      </c>
-      <c r="H4">
-        <v>12990</v>
-      </c>
-      <c r="I4">
-        <v>5</v>
-      </c>
-      <c r="J4">
-        <v>12340.5</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Intermediate</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Quality Assurance Master</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Priya Nair</v>
-      </c>
-      <c r="C5" t="str">
-        <v>QA automation and testing</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Quality</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-05-01</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2026-05-15</v>
-      </c>
-      <c r="G5">
-        <v>40</v>
-      </c>
-      <c r="H5">
-        <v>9990</v>
-      </c>
-      <c r="I5">
-        <v>15</v>
-      </c>
-      <c r="J5">
-        <v>8491.5</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Advanced</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Project Management Pro</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Amit Shah</v>
-      </c>
-      <c r="C6" t="str">
-        <v>PM skills and tools</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Project</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-06-01</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2026-06-12</v>
-      </c>
-      <c r="G6">
-        <v>24</v>
-      </c>
-      <c r="H6">
-        <v>10990</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>9671.2</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Intermediate</v>
+      <c r="Q2">
+        <v>450</v>
+      </c>
+      <c r="R2">
+        <v>650</v>
+      </c>
+      <c r="S2">
+        <v>10</v>
+      </c>
+      <c r="T2">
+        <v>585</v>
+      </c>
+      <c r="U2">
+        <v>450</v>
+      </c>
+      <c r="V2">
+        <v>10</v>
+      </c>
+      <c r="W2">
+        <v>405</v>
+      </c>
+      <c r="X2">
+        <v>40000</v>
+      </c>
+      <c r="Y2">
+        <v>10</v>
+      </c>
+      <c r="Z2">
+        <v>36000</v>
+      </c>
+      <c r="AA2">
+        <v>700</v>
+      </c>
+      <c r="AB2">
+        <v>10</v>
+      </c>
+      <c r="AC2">
+        <v>630</v>
+      </c>
+      <c r="AD2">
+        <v>680</v>
+      </c>
+      <c r="AE2">
+        <v>10</v>
+      </c>
+      <c r="AF2">
+        <v>612</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
brochure drive link upload to db and show in view edit and add delete functionality
</commit_message>
<xml_diff>
--- a/public/course-import-template.xlsx
+++ b/public/course-import-template.xlsx
@@ -397,161 +397,165 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AG2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="18.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="18.83203125" customWidth="1"/>
-    <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" width="18.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" customWidth="1"/>
-    <col min="24" max="24" width="18.83203125" customWidth="1"/>
-    <col min="25" max="25" width="18.83203125" customWidth="1"/>
-    <col min="26" max="26" width="18.83203125" customWidth="1"/>
-    <col min="27" max="27" width="18.83203125" customWidth="1"/>
-    <col min="28" max="28" width="18.83203125" customWidth="1"/>
-    <col min="29" max="29" width="18.83203125" customWidth="1"/>
-    <col min="30" max="30" width="18.83203125" customWidth="1"/>
-    <col min="31" max="31" width="18.83203125" customWidth="1"/>
-    <col min="32" max="32" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="15.83203125" customWidth="1"/>
+    <col min="15" max="15" width="40.83203125" customWidth="1"/>
+    <col min="16" max="16" width="15.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="15.83203125" customWidth="1"/>
+    <col min="19" max="19" width="15.83203125" customWidth="1"/>
+    <col min="20" max="20" width="15.83203125" customWidth="1"/>
+    <col min="21" max="21" width="15.83203125" customWidth="1"/>
+    <col min="22" max="22" width="15.83203125" customWidth="1"/>
+    <col min="23" max="23" width="15.83203125" customWidth="1"/>
+    <col min="24" max="24" width="15.83203125" customWidth="1"/>
+    <col min="25" max="25" width="15.83203125" customWidth="1"/>
+    <col min="26" max="26" width="15.83203125" customWidth="1"/>
+    <col min="27" max="27" width="15.83203125" customWidth="1"/>
+    <col min="28" max="28" width="15.83203125" customWidth="1"/>
+    <col min="29" max="29" width="15.83203125" customWidth="1"/>
+    <col min="30" max="30" width="15.83203125" customWidth="1"/>
+    <col min="31" max="31" width="15.83203125" customWidth="1"/>
+    <col min="32" max="32" width="15.83203125" customWidth="1"/>
+    <col min="33" max="33" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Course Name</v>
+        <v>courseName</v>
       </c>
       <c r="B1" t="str">
-        <v>Mentor</v>
+        <v>description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>mentor</v>
       </c>
       <c r="D1" t="str">
-        <v>Service Type</v>
+        <v>serviceType</v>
       </c>
       <c r="E1" t="str">
-        <v>Level</v>
+        <v>difficultyLevel</v>
       </c>
       <c r="F1" t="str">
-        <v>Start Date</v>
+        <v>startDate</v>
       </c>
       <c r="G1" t="str">
-        <v>End Date</v>
+        <v>endDate</v>
       </c>
       <c r="H1" t="str">
-        <v>Duration</v>
+        <v>duration</v>
       </c>
       <c r="I1" t="str">
-        <v>Language</v>
+        <v>language</v>
       </c>
       <c r="J1" t="str">
-        <v>Start Time</v>
+        <v>startTime</v>
       </c>
       <c r="K1" t="str">
-        <v>End Time</v>
+        <v>endTime</v>
       </c>
       <c r="L1" t="str">
-        <v>Batch Type</v>
+        <v>batchType</v>
       </c>
       <c r="M1" t="str">
-        <v>Course Type</v>
+        <v>courseType</v>
       </c>
       <c r="N1" t="str">
-        <v>Address</v>
+        <v>address</v>
       </c>
       <c r="O1" t="str">
-        <v>Fee (USA)</v>
+        <v>brochure</v>
       </c>
       <c r="P1" t="str">
-        <v>Discount (USA)</v>
+        <v>feeUSA</v>
       </c>
       <c r="Q1" t="str">
-        <v>Price (USA)</v>
+        <v>discountUSA</v>
       </c>
       <c r="R1" t="str">
-        <v>Fee (Canadian)</v>
+        <v>priceUSA</v>
       </c>
       <c r="S1" t="str">
-        <v>Discount (Canadian)</v>
+        <v>feeCanadian</v>
       </c>
       <c r="T1" t="str">
-        <v>Price (Canadian)</v>
+        <v>discountCanadian</v>
       </c>
       <c r="U1" t="str">
-        <v>Fee (Europe)</v>
+        <v>priceCanadian</v>
       </c>
       <c r="V1" t="str">
-        <v>Discount (Europe)</v>
+        <v>feeEurope</v>
       </c>
       <c r="W1" t="str">
-        <v>Price (Europe)</v>
+        <v>discountEurope</v>
       </c>
       <c r="X1" t="str">
-        <v>Fee (India)</v>
+        <v>priceEurope</v>
       </c>
       <c r="Y1" t="str">
-        <v>Discount (India)</v>
+        <v>feeIndia</v>
       </c>
       <c r="Z1" t="str">
-        <v>Price (India)</v>
+        <v>discountIndia</v>
       </c>
       <c r="AA1" t="str">
-        <v>Fee (Australia)</v>
+        <v>priceIndia</v>
       </c>
       <c r="AB1" t="str">
-        <v>Discount (Australia)</v>
+        <v>feeAustralia</v>
       </c>
       <c r="AC1" t="str">
-        <v>Price (Australia)</v>
+        <v>discountAustralia</v>
       </c>
       <c r="AD1" t="str">
-        <v>Fee (Singapore)</v>
+        <v>priceAustralia</v>
       </c>
       <c r="AE1" t="str">
-        <v>Discount (Singapore)</v>
+        <v>feeSingapore</v>
       </c>
       <c r="AF1" t="str">
-        <v>Price (Singapore)</v>
+        <v>discountSingapore</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>priceSingapore</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Advanced Python</v>
+        <v>Sample Course 101</v>
       </c>
       <c r="B2" t="str">
+        <v>A comprehensive introduction to the course topic.</v>
+      </c>
+      <c r="C2" t="str">
         <v>John Doe</v>
       </c>
-      <c r="C2" t="str">
-        <v>Comprehensive Python course covering advanced topics.</v>
-      </c>
       <c r="D2" t="str">
-        <v>Agile</v>
+        <v>Generative AI</v>
       </c>
       <c r="E2" t="str">
-        <v>Advanced</v>
+        <v>Beginner</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-03-01</v>
+        <v>2024-01-01</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-03-30</v>
+        <v>2024-01-31</v>
       </c>
       <c r="H2">
         <v>30</v>
@@ -574,64 +578,67 @@
       <c r="N2" t="str">
         <v/>
       </c>
-      <c r="O2">
+      <c r="O2" t="str">
+        <v>https://example.com/public-brochure.pdf</v>
+      </c>
+      <c r="P2">
         <v>500</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>10</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>450</v>
       </c>
-      <c r="R2">
-        <v>650</v>
-      </c>
       <c r="S2">
+        <v>600</v>
+      </c>
+      <c r="T2">
         <v>10</v>
       </c>
-      <c r="T2">
-        <v>585</v>
-      </c>
       <c r="U2">
+        <v>540</v>
+      </c>
+      <c r="V2">
         <v>450</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>10</v>
       </c>
-      <c r="W2">
+      <c r="X2">
         <v>405</v>
       </c>
-      <c r="X2">
-        <v>40000</v>
-      </c>
       <c r="Y2">
+        <v>5000</v>
+      </c>
+      <c r="Z2">
         <v>10</v>
       </c>
-      <c r="Z2">
-        <v>36000</v>
-      </c>
       <c r="AA2">
+        <v>4500</v>
+      </c>
+      <c r="AB2">
         <v>700</v>
       </c>
-      <c r="AB2">
+      <c r="AC2">
         <v>10</v>
       </c>
-      <c r="AC2">
+      <c r="AD2">
         <v>630</v>
       </c>
-      <c r="AD2">
-        <v>680</v>
-      </c>
       <c r="AE2">
+        <v>800</v>
+      </c>
+      <c r="AF2">
         <v>10</v>
       </c>
-      <c r="AF2">
-        <v>612</v>
+      <c r="AG2">
+        <v>720</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AG2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Ganesh] Update courseController.ts and admin navabr and dashboard
</commit_message>
<xml_diff>
--- a/public/course-import-template.xlsx
+++ b/public/course-import-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Courses" sheetId="1" r:id="rId1"/>
+    <sheet name="Import Template" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,42 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AG2"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" customWidth="1"/>
-    <col min="13" max="13" width="15.83203125" customWidth="1"/>
-    <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="40.83203125" customWidth="1"/>
-    <col min="16" max="16" width="15.83203125" customWidth="1"/>
-    <col min="17" max="17" width="15.83203125" customWidth="1"/>
-    <col min="18" max="18" width="15.83203125" customWidth="1"/>
-    <col min="19" max="19" width="15.83203125" customWidth="1"/>
-    <col min="20" max="20" width="15.83203125" customWidth="1"/>
-    <col min="21" max="21" width="15.83203125" customWidth="1"/>
-    <col min="22" max="22" width="15.83203125" customWidth="1"/>
-    <col min="23" max="23" width="15.83203125" customWidth="1"/>
-    <col min="24" max="24" width="15.83203125" customWidth="1"/>
-    <col min="25" max="25" width="15.83203125" customWidth="1"/>
-    <col min="26" max="26" width="15.83203125" customWidth="1"/>
-    <col min="27" max="27" width="15.83203125" customWidth="1"/>
-    <col min="28" max="28" width="15.83203125" customWidth="1"/>
-    <col min="29" max="29" width="15.83203125" customWidth="1"/>
-    <col min="30" max="30" width="15.83203125" customWidth="1"/>
-    <col min="31" max="31" width="15.83203125" customWidth="1"/>
-    <col min="32" max="32" width="15.83203125" customWidth="1"/>
-    <col min="33" max="33" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:AJ2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -478,60 +443,69 @@
         <v>address</v>
       </c>
       <c r="O1" t="str">
+        <v>maxParticipants</v>
+      </c>
+      <c r="P1" t="str">
+        <v>planAvailable</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>isActive</v>
+      </c>
+      <c r="R1" t="str">
         <v>brochure</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>feeUSA</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>discountUSA</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>priceUSA</v>
       </c>
-      <c r="S1" t="str">
-        <v>feeCanadian</v>
-      </c>
-      <c r="T1" t="str">
-        <v>discountCanadian</v>
-      </c>
-      <c r="U1" t="str">
-        <v>priceCanadian</v>
-      </c>
       <c r="V1" t="str">
+        <v>feeCanada</v>
+      </c>
+      <c r="W1" t="str">
+        <v>discountCanada</v>
+      </c>
+      <c r="X1" t="str">
+        <v>priceCanada</v>
+      </c>
+      <c r="Y1" t="str">
         <v>feeEurope</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Z1" t="str">
         <v>discountEurope</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AA1" t="str">
         <v>priceEurope</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AB1" t="str">
         <v>feeIndia</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AC1" t="str">
         <v>discountIndia</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>priceIndia</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
         <v>feeAustralia</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AF1" t="str">
         <v>discountAustralia</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AG1" t="str">
         <v>priceAustralia</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AH1" t="str">
         <v>feeSingapore</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AI1" t="str">
         <v>discountSingapore</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AJ1" t="str">
         <v>priceSingapore</v>
       </c>
     </row>
@@ -552,10 +526,10 @@
         <v>Beginner</v>
       </c>
       <c r="F2" t="str">
-        <v>2024-01-01</v>
+        <v>2026-05-01</v>
       </c>
       <c r="G2" t="str">
-        <v>2024-01-31</v>
+        <v>2026-05-31</v>
       </c>
       <c r="H2">
         <v>30</v>
@@ -570,7 +544,7 @@
         <v>12:00</v>
       </c>
       <c r="L2" t="str">
-        <v>Weekdays</v>
+        <v>Weekend</v>
       </c>
       <c r="M2" t="str">
         <v>Online</v>
@@ -578,67 +552,76 @@
       <c r="N2" t="str">
         <v/>
       </c>
-      <c r="O2" t="str">
+      <c r="O2">
+        <v>30</v>
+      </c>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R2" t="str">
         <v>https://example.com/public-brochure.pdf</v>
       </c>
-      <c r="P2">
+      <c r="S2">
         <v>500</v>
-      </c>
-      <c r="Q2">
-        <v>10</v>
-      </c>
-      <c r="R2">
-        <v>450</v>
-      </c>
-      <c r="S2">
-        <v>600</v>
       </c>
       <c r="T2">
         <v>10</v>
       </c>
       <c r="U2">
-        <v>540</v>
+        <v>450</v>
       </c>
       <c r="V2">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="W2">
         <v>10</v>
       </c>
       <c r="X2">
-        <v>405</v>
+        <v>540</v>
       </c>
       <c r="Y2">
-        <v>5000</v>
+        <v>450</v>
       </c>
       <c r="Z2">
         <v>10</v>
       </c>
       <c r="AA2">
-        <v>4500</v>
+        <v>405</v>
       </c>
       <c r="AB2">
-        <v>700</v>
+        <v>5000</v>
       </c>
       <c r="AC2">
         <v>10</v>
       </c>
       <c r="AD2">
-        <v>630</v>
+        <v>4500</v>
       </c>
       <c r="AE2">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="AF2">
         <v>10</v>
       </c>
       <c r="AG2">
+        <v>630</v>
+      </c>
+      <c r="AH2">
+        <v>800</v>
+      </c>
+      <c r="AI2">
+        <v>10</v>
+      </c>
+      <c r="AJ2">
         <v>720</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AG2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AJ2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>